<commit_message>
Fit all six columns on screen without sideways scrolling
The board now breaks out of the 1300px text column to the window edges,
capped at 1780px on very wide screens and returning to the normal column
below 900px. Its minimum width drops from 1420 to 1200 now that the
keywords are shorter.

Shortened 47 entry labels that were wrapping to two lines. At a 1440px
window every column is visible at 223px wide with no wrapped chip and no
horizontal scroll. Band heights rebalanced 1 : 1.1 : 1.5 for the taller
dry row.

Also add the viewport meta tag, without which phones laid the page out at
980px and none of the mobile breakpoints fired.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/releaf-six-minds-en.xlsx
+++ b/releaf-six-minds-en.xlsx
@@ -600,7 +600,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phenotype: germination, root, weight</t>
+          <t xml:space="preserve">Germination, root, weight</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dr. Brophy · must pass the membrane</t>
+          <t xml:space="preserve">Brophy · must pass the membrane</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1869,7 +1869,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Compared against proline, trehalose, ectoine</t>
+          <t xml:space="preserve">Against proline and ectoine</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2010,7 +2010,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Codon optimisation, shared with M3</t>
+          <t xml:space="preserve">Codon optimisation, shared</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2151,7 +2151,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dr. Brophy · light in, containment first</t>
+          <t xml:space="preserve">Brophy · light in, contain first</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2339,7 +2339,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t xml:space="preserve">pNW33N-L2 (sfGFP) shuttle vector</t>
+          <t xml:space="preserve">pNW33N-L2 shuttle vector</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2527,7 +2527,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fold change: 535 against 670 nm</t>
+          <t xml:space="preserve">Fold change 535 / 670 nm</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2715,7 +2715,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Characterise each promoter alone</t>
+          <t xml:space="preserve">Each promoter alone first</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2903,7 +2903,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cello logic and where you overrode it</t>
+          <t xml:space="preserve">Cello, and your overrides</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3185,7 +3185,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Biotech Expo · aeration and modularity</t>
+          <t xml:space="preserve">Expo · aeration, modularity</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3326,7 +3326,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t xml:space="preserve">Containment: no colonies outside</t>
+          <t xml:space="preserve">No colonies outside</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3373,7 +3373,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t xml:space="preserve">Passage: His-tag detected outside</t>
+          <t xml:space="preserve">His-tag detected outside</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -3467,7 +3467,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t xml:space="preserve">Foaming and resting-cell operation</t>
+          <t xml:space="preserve">Foaming, resting cells</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -3749,7 +3749,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t xml:space="preserve">Valve pressure across the membrane</t>
+          <t xml:space="preserve">Valve pressure across membrane</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -3796,7 +3796,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reynolds number and flow regime</t>
+          <t xml:space="preserve">Reynolds and flow regime</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -3843,7 +3843,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mass transfer, heat, oxygen at scale</t>
+          <t xml:space="preserve">Mass transfer at scale</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -4031,7 +4031,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t xml:space="preserve">Control stack: Arduino, pump, sensors</t>
+          <t xml:space="preserve">Arduino, pump, sensors</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -4078,7 +4078,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t xml:space="preserve">Three independent containment layers</t>
+          <t xml:space="preserve">Three containment layers</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t xml:space="preserve">Membrane wear and service schedule</t>
+          <t xml:space="preserve">Membrane wear, servicing</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -4172,7 +4172,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t xml:space="preserve">Build files: BOM, firmware, enclosure</t>
+          <t xml:space="preserve">BOM, firmware, enclosure</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -4266,7 +4266,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t xml:space="preserve">What the team built against bought</t>
+          <t xml:space="preserve">Built against bought</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -4313,7 +4313,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t xml:space="preserve">Version milestones and enclosure</t>
+          <t xml:space="preserve">Version milestones</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -4454,7 +4454,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t xml:space="preserve">World Veg · sustainable, not organic</t>
+          <t xml:space="preserve">World Veg · not organic</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -4689,7 +4689,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t xml:space="preserve">The numbers behind the problem</t>
+          <t xml:space="preserve">The problem in numbers</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -4783,7 +4783,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tests the biostimulant path requires</t>
+          <t xml:space="preserve">Biostimulant path tests</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -4830,7 +4830,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t xml:space="preserve">The biopesticide battery avoided</t>
+          <t xml:space="preserve">Biopesticide tests avoided</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -4877,7 +4877,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t xml:space="preserve">Containment evidence for a regulator</t>
+          <t xml:space="preserve">Evidence a regulator accepts</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t xml:space="preserve">Farm size against climate volatility</t>
+          <t xml:space="preserve">Farm size × volatility</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -4971,7 +4971,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interpolation method and uncertainty</t>
+          <t xml:space="preserve">Interpolation, uncertainty</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -5018,7 +5018,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fertilizer Act against Pesticide Act</t>
+          <t xml:space="preserve">Fertilizer vs Pesticide Act</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -5065,7 +5065,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t xml:space="preserve">30 days against several years</t>
+          <t xml:space="preserve">30 days vs years</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contained use against release</t>
+          <t xml:space="preserve">Contained use vs release</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -5159,7 +5159,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t xml:space="preserve">Attribution: students against collaborators</t>
+          <t xml:space="preserve">Attribution split</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
@@ -5488,7 +5488,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yield per cartridge run</t>
+          <t xml:space="preserve">Yield per cartridge</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -5535,7 +5535,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cartridge lifetime under load</t>
+          <t xml:space="preserve">Cartridge lifetime</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -5629,7 +5629,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t xml:space="preserve">Map to addressable market</t>
+          <t xml:space="preserve">Addressable market</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -5676,7 +5676,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t xml:space="preserve">Device cheap, cartridge recurring</t>
+          <t xml:space="preserve">Device and cartridge split</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -5723,7 +5723,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t xml:space="preserve">Market sequence and its reasons</t>
+          <t xml:space="preserve">Market sequence</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -5770,7 +5770,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t xml:space="preserve">Patent against trade secret</t>
+          <t xml:space="preserve">Patent vs trade secret</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -5817,7 +5817,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cartridge against seasonal fungicide</t>
+          <t xml:space="preserve">Cartridge vs fungicide</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -5958,7 +5958,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t xml:space="preserve">Value per device per season</t>
+          <t xml:space="preserve">Value per device-season</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -6005,7 +6005,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cost of goods per cartridge</t>
+          <t xml:space="preserve">Cost per cartridge</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
@@ -6052,7 +6052,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gross margin and the price floor</t>
+          <t xml:space="preserve">Margin and price floor</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modular cassette as a platform</t>
+          <t xml:space="preserve">Cassette as a platform</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -6146,7 +6146,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freedom to operate on the parts</t>
+          <t xml:space="preserve">Freedom to operate</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -6193,7 +6193,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t xml:space="preserve">Funding stages and their evidence</t>
+          <t xml:space="preserve">Funding stages</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -6240,7 +6240,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t xml:space="preserve">Competitors and the gap we sit in</t>
+          <t xml:space="preserve">Competitors and the gap</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">

</xml_diff>